<commit_message>
photo enlarge and synonyms in search bar
</commit_message>
<xml_diff>
--- a/test_review.xlsx
+++ b/test_review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\emanual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5123764-8D5D-4240-8EBC-5BA80F4E3ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{154CE664-AAAE-412B-92CB-187E4A97BA44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7270" uniqueCount="2520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7270" uniqueCount="2523">
   <si>
     <t>Test ID</t>
   </si>
@@ -8503,6 +8503,21 @@
       </rPr>
       <t xml:space="preserve"> to enter staff mode and allow display of "Lab handling"</t>
     </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>CMS Name
+(include in search index)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Label Name
+(include in search index)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Synonyms
+(include in search index)</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -8698,13 +8713,13 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -9027,35 +9042,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="16" t="s">
         <v>2518</v>
       </c>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="16" t="s">
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="17" t="s">
         <v>2517</v>
       </c>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="15" t="s">
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="16" t="s">
         <v>2519</v>
       </c>
-      <c r="K1" s="15"/>
+      <c r="K1" s="16"/>
     </row>
     <row r="2" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>2520</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>2521</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
+        <v>2522</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>4</v>

</xml_diff>